<commit_message>
data: tighten debt package reconciliation
</commit_message>
<xml_diff>
--- a/docs/Raw Data/Debt/government-debt-annual/government-debt-review.xlsx
+++ b/docs/Raw Data/Debt/government-debt-annual/government-debt-review.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R4ddcf949bb214ecb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock" sheetId="2" r:id="Rd4c962bc86914099"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interest rates" sheetId="3" r:id="R74606cb7ac7a4109"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actual service" sheetId="4" r:id="Rbfcfbb143116401f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast service" sheetId="5" r:id="R2191c8c5894640d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2019-2022 controls" sheetId="6" r:id="R28b4c492002845f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" r:id="Reffd7b71285c49bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="Rb67b0f9f0cd440ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock" sheetId="2" r:id="R48b01bf2e50d40ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interest rates" sheetId="3" r:id="Rc657fcdfa11344a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actual service" sheetId="4" r:id="R6ba584c233084d12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast service" sheetId="5" r:id="R05977a7b15b14abb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2019-2022 controls" sheetId="6" r:id="R8ad5b16b670847fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" r:id="Rb9967bbf09984ebd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2709,7 +2709,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re45b865978874607"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83e645bf05124415"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3234,19 +3234,19 @@
         <x:v>not_found_in_reviewed_sources</x:v>
       </x:c>
       <x:c r="H13" s="38" t="str">
-        <x:v>mof_monthly_debt_report_2026_07</x:v>
+        <x:v>mof_debt_strategy_2019_2021</x:v>
       </x:c>
       <x:c r="I13" s="38" t="str">
-        <x:v>Reviewed official source set</x:v>
+        <x:v>Table 2: Weighted Average Interest Rates on General Government Domestic and External Debt</x:v>
       </x:c>
       <x:c r="J13" s="38" t="str">
-        <x:v>No comparable source row</x:v>
+        <x:v>External Debt / Eurobond</x:v>
       </x:c>
       <x:c r="K13" s="38" t="str">
         <x:v>% p.a.</x:v>
       </x:c>
       <x:c r="L13" s="50" t="str">
-        <x:v>The reviewed component table excludes the Eurobond, so it is not normalized as the full External Government Debt portfolio rate.</x:v>
+        <x:v>The reviewed component table reports External Debt and Eurobond separately, so the External Debt row is not normalized as the full External Government Debt portfolio rate.</x:v>
       </x:c>
       <x:c r="M13" s="44" t="n">
         <x:v>46266</x:v>
@@ -3355,13 +3355,13 @@
         <x:v>not_found_in_reviewed_sources</x:v>
       </x:c>
       <x:c r="H16" s="38" t="str">
-        <x:v>mof_monthly_debt_report_2026_07</x:v>
+        <x:v>mof_debt_strategy_2022_2025</x:v>
       </x:c>
       <x:c r="I16" s="38" t="str">
-        <x:v>Reviewed official source set</x:v>
+        <x:v>Table 4.1: Weighted Average Interest Rates on the General Government Domestic and External Debt Portfolios</x:v>
       </x:c>
       <x:c r="J16" s="38" t="str">
-        <x:v>No comparable source row</x:v>
+        <x:v>External Debt (excludes the Eurobond)</x:v>
       </x:c>
       <x:c r="K16" s="38" t="str">
         <x:v>% p.a.</x:v>
@@ -3476,13 +3476,13 @@
         <x:v>not_found_in_reviewed_sources</x:v>
       </x:c>
       <x:c r="H19" s="38" t="str">
-        <x:v>mof_monthly_debt_report_2026_07</x:v>
+        <x:v>mof_debt_strategy_2022_2025</x:v>
       </x:c>
       <x:c r="I19" s="38" t="str">
-        <x:v>Reviewed official source set</x:v>
+        <x:v>Table 4.1: Weighted Average Interest Rates on the General Government Domestic and External Debt Portfolios</x:v>
       </x:c>
       <x:c r="J19" s="38" t="str">
-        <x:v>No comparable source row</x:v>
+        <x:v>External Debt (excludes the Eurobond)</x:v>
       </x:c>
       <x:c r="K19" s="38" t="str">
         <x:v>% p.a.</x:v>
@@ -4108,7 +4108,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R057860cd4b72495b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2022e87912d143b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5826,7 +5826,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e5fec86f57a44e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7efbaf81ab64b5c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5950,7 +5950,7 @@
         <x:v>1613.8312668464</x:v>
       </x:c>
       <x:c r="L2" s="40" t="n">
-        <x:v>5160.8401105122</x:v>
+        <x:v>5160.8291105122</x:v>
       </x:c>
       <x:c r="M2" s="37" t="str">
         <x:v>projection_existing_portfolio</x:v>
@@ -6127,7 +6127,7 @@
         <x:v>1467.509703504</x:v>
       </x:c>
       <x:c r="L5" s="41" t="n">
-        <x:v>4388.4298625336</x:v>
+        <x:v>4388.3808625336</x:v>
       </x:c>
       <x:c r="M5" s="38" t="str">
         <x:v>projection_existing_portfolio</x:v>
@@ -6304,7 +6304,7 @@
         <x:v>1227.3514824798</x:v>
       </x:c>
       <x:c r="L8" s="41" t="n">
-        <x:v>5480.0999487871</x:v>
+        <x:v>5480.0889487871</x:v>
       </x:c>
       <x:c r="M8" s="38" t="str">
         <x:v>projection_existing_portfolio</x:v>
@@ -6481,7 +6481,7 @@
         <x:v>1060.4892183288</x:v>
       </x:c>
       <x:c r="L11" s="41" t="n">
-        <x:v>3879.0845121293</x:v>
+        <x:v>3879.1105121293</x:v>
       </x:c>
       <x:c r="M11" s="38" t="str">
         <x:v>projection_existing_portfolio</x:v>
@@ -6658,7 +6658,7 @@
         <x:v>831.518328841</x:v>
       </x:c>
       <x:c r="L14" s="41" t="n">
-        <x:v>3720.0654420485</x:v>
+        <x:v>3720.0164420485</x:v>
       </x:c>
       <x:c r="M14" s="38" t="str">
         <x:v>projection_existing_portfolio</x:v>
@@ -6803,7 +6803,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c4ee26d88eb4981"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R122b4589500a4b6c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6941,7 +6941,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d1d0da6f78f4be7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25fed8be1a234af4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7159,13 +7159,13 @@
         <x:v>2022</x:v>
       </x:c>
       <x:c r="N4" s="34" t="n">
-        <x:v>2020</x:v>
+        <x:v>2015</x:v>
       </x:c>
       <x:c r="O4" s="34" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="P4" s="50" t="str">
-        <x:v>External Government Debt principal and interest paid for 2020-2022; overlapping stock is a control.</x:v>
+        <x:v>External Government Debt principal and interest paid for 2020-2022; Government Debt stock is used as an overlap control for 2015-2022.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="64" customHeight="1">
@@ -7590,8 +7590,8 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ed66c3a07054c73"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4edc2d1e1ebe4c3c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7b8033fea534d6b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2da97088447d48a2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>